<commit_message>
revise test report details
</commit_message>
<xml_diff>
--- a/Test_Report.xlsx
+++ b/Test_Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbookpro/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{79125C0D-A31B-064B-8E3D-1A3692EC0D5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C1757D45-FEB7-6048-B68F-54023ADB741D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{170E7E5C-781E-774B-8F68-80F2A3A7B57F}"/>
   </bookViews>
@@ -2959,7 +2959,7 @@
     <col min="4" max="4" width="15.140625" customWidth="1"/>
     <col min="6" max="6" width="26.7109375" customWidth="1"/>
     <col min="7" max="7" width="14.85546875" customWidth="1"/>
-    <col min="8" max="8" width="16.140625" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
     <col min="9" max="9" width="10.5703125" customWidth="1"/>
     <col min="16" max="16" width="11.140625" customWidth="1"/>
   </cols>
@@ -2985,7 +2985,7 @@
       <c r="B2" s="41"/>
       <c r="C2" s="30"/>
       <c r="D2" s="42">
-        <v>46129</v>
+        <v>46098</v>
       </c>
       <c r="E2" s="41"/>
       <c r="F2" s="41"/>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="B5" s="30"/>
       <c r="C5" s="42">
-        <v>46124</v>
+        <v>46093</v>
       </c>
       <c r="D5" s="41"/>
       <c r="E5" s="30"/>
@@ -3046,7 +3046,7 @@
         <v>27</v>
       </c>
       <c r="G5" s="42">
-        <v>46129</v>
+        <v>46099</v>
       </c>
       <c r="H5" s="41"/>
       <c r="I5" s="41"/>

</xml_diff>